<commit_message>
v1.2.0: regenerated reports and figures, README and requirements updated for the removed limitations
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AU7pCHF2so4EmjE8rSm1Ka
</commit_message>
<xml_diff>
--- a/excel/gtperf_site_tool.xlsx
+++ b/excel/gtperf_site_tool.xlsx
@@ -1035,23 +1035,23 @@
         </is>
       </c>
       <c r="D21" s="11">
-        <f>1+FORECAST(D7,OFFSET(INLET_POWER,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D10/D16</f>
+        <f>1+FORECAST(D7,OFFSET(INLET_POWER,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D10</f>
         <v/>
       </c>
       <c r="E21" s="11">
-        <f>1+FORECAST(E7,OFFSET(INLET_POWER,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E10/E16</f>
+        <f>1+FORECAST(E7,OFFSET(INLET_POWER,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E10</f>
         <v/>
       </c>
       <c r="F21" s="11">
-        <f>1+FORECAST(F7,OFFSET(INLET_POWER,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F10/F16</f>
+        <f>1+FORECAST(F7,OFFSET(INLET_POWER,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F10</f>
         <v/>
       </c>
       <c r="G21" s="11">
-        <f>1+FORECAST(G7,OFFSET(INLET_POWER,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G10/G16</f>
+        <f>1+FORECAST(G7,OFFSET(INLET_POWER,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G10</f>
         <v/>
       </c>
       <c r="H21" s="11">
-        <f>1+FORECAST(H7,OFFSET(INLET_POWER,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H10/H16</f>
+        <f>1+FORECAST(H7,OFFSET(INLET_POWER,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H10</f>
         <v/>
       </c>
     </row>
@@ -1067,23 +1067,23 @@
         </is>
       </c>
       <c r="D22" s="11">
-        <f>1+FORECAST(D7,OFFSET(EXHAUST_POWER,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D11/D16</f>
+        <f>1+FORECAST(D7,OFFSET(EXHAUST_POWER,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D11</f>
         <v/>
       </c>
       <c r="E22" s="11">
-        <f>1+FORECAST(E7,OFFSET(EXHAUST_POWER,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E11/E16</f>
+        <f>1+FORECAST(E7,OFFSET(EXHAUST_POWER,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E11</f>
         <v/>
       </c>
       <c r="F22" s="11">
-        <f>1+FORECAST(F7,OFFSET(EXHAUST_POWER,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F11/F16</f>
+        <f>1+FORECAST(F7,OFFSET(EXHAUST_POWER,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F11</f>
         <v/>
       </c>
       <c r="G22" s="11">
-        <f>1+FORECAST(G7,OFFSET(EXHAUST_POWER,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G11/G16</f>
+        <f>1+FORECAST(G7,OFFSET(EXHAUST_POWER,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G11</f>
         <v/>
       </c>
       <c r="H22" s="11">
-        <f>1+FORECAST(H7,OFFSET(EXHAUST_POWER,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H11/H16</f>
+        <f>1+FORECAST(H7,OFFSET(EXHAUST_POWER,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H11</f>
         <v/>
       </c>
     </row>
@@ -1195,23 +1195,23 @@
         </is>
       </c>
       <c r="D26" s="11">
-        <f>1+FORECAST(D7,OFFSET(INLET_HEAT_RATE,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D10/D16</f>
+        <f>1+FORECAST(D7,OFFSET(INLET_HEAT_RATE,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D10</f>
         <v/>
       </c>
       <c r="E26" s="11">
-        <f>1+FORECAST(E7,OFFSET(INLET_HEAT_RATE,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E10/E16</f>
+        <f>1+FORECAST(E7,OFFSET(INLET_HEAT_RATE,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E10</f>
         <v/>
       </c>
       <c r="F26" s="11">
-        <f>1+FORECAST(F7,OFFSET(INLET_HEAT_RATE,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F10/F16</f>
+        <f>1+FORECAST(F7,OFFSET(INLET_HEAT_RATE,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F10</f>
         <v/>
       </c>
       <c r="G26" s="11">
-        <f>1+FORECAST(G7,OFFSET(INLET_HEAT_RATE,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G10/G16</f>
+        <f>1+FORECAST(G7,OFFSET(INLET_HEAT_RATE,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G10</f>
         <v/>
       </c>
       <c r="H26" s="11">
-        <f>1+FORECAST(H7,OFFSET(INLET_HEAT_RATE,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H10/H16</f>
+        <f>1+FORECAST(H7,OFFSET(INLET_HEAT_RATE,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H10</f>
         <v/>
       </c>
     </row>
@@ -1227,23 +1227,23 @@
         </is>
       </c>
       <c r="D27" s="11">
-        <f>1+FORECAST(D7,OFFSET(EXHAUST_HEAT_RATE,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D11/D16</f>
+        <f>1+FORECAST(D7,OFFSET(EXHAUST_HEAT_RATE,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D11</f>
         <v/>
       </c>
       <c r="E27" s="11">
-        <f>1+FORECAST(E7,OFFSET(EXHAUST_HEAT_RATE,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E11/E16</f>
+        <f>1+FORECAST(E7,OFFSET(EXHAUST_HEAT_RATE,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E11</f>
         <v/>
       </c>
       <c r="F27" s="11">
-        <f>1+FORECAST(F7,OFFSET(EXHAUST_HEAT_RATE,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F11/F16</f>
+        <f>1+FORECAST(F7,OFFSET(EXHAUST_HEAT_RATE,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F11</f>
         <v/>
       </c>
       <c r="G27" s="11">
-        <f>1+FORECAST(G7,OFFSET(EXHAUST_HEAT_RATE,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G11/G16</f>
+        <f>1+FORECAST(G7,OFFSET(EXHAUST_HEAT_RATE,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G11</f>
         <v/>
       </c>
       <c r="H27" s="11">
-        <f>1+FORECAST(H7,OFFSET(EXHAUST_HEAT_RATE,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H11/H16</f>
+        <f>1+FORECAST(H7,OFFSET(EXHAUST_HEAT_RATE,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H11</f>
         <v/>
       </c>
     </row>
@@ -1355,23 +1355,23 @@
         </is>
       </c>
       <c r="D31" s="11">
-        <f>1+FORECAST(D7,OFFSET(INLET_EXHAUST_FLOW,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D10/D16</f>
+        <f>1+FORECAST(D7,OFFSET(INLET_EXHAUST_FLOW,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D10</f>
         <v/>
       </c>
       <c r="E31" s="11">
-        <f>1+FORECAST(E7,OFFSET(INLET_EXHAUST_FLOW,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E10/E16</f>
+        <f>1+FORECAST(E7,OFFSET(INLET_EXHAUST_FLOW,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E10</f>
         <v/>
       </c>
       <c r="F31" s="11">
-        <f>1+FORECAST(F7,OFFSET(INLET_EXHAUST_FLOW,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F10/F16</f>
+        <f>1+FORECAST(F7,OFFSET(INLET_EXHAUST_FLOW,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F10</f>
         <v/>
       </c>
       <c r="G31" s="11">
-        <f>1+FORECAST(G7,OFFSET(INLET_EXHAUST_FLOW,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G10/G16</f>
+        <f>1+FORECAST(G7,OFFSET(INLET_EXHAUST_FLOW,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G10</f>
         <v/>
       </c>
       <c r="H31" s="11">
-        <f>1+FORECAST(H7,OFFSET(INLET_EXHAUST_FLOW,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H10/H16</f>
+        <f>1+FORECAST(H7,OFFSET(INLET_EXHAUST_FLOW,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H10</f>
         <v/>
       </c>
     </row>
@@ -1387,23 +1387,23 @@
         </is>
       </c>
       <c r="D32" s="11">
-        <f>1+FORECAST(D7,OFFSET(EXHAUST_EXHAUST_FLOW,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D11/D16</f>
+        <f>1+FORECAST(D7,OFFSET(EXHAUST_EXHAUST_FLOW,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D11</f>
         <v/>
       </c>
       <c r="E32" s="11">
-        <f>1+FORECAST(E7,OFFSET(EXHAUST_EXHAUST_FLOW,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E11/E16</f>
+        <f>1+FORECAST(E7,OFFSET(EXHAUST_EXHAUST_FLOW,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E11</f>
         <v/>
       </c>
       <c r="F32" s="11">
-        <f>1+FORECAST(F7,OFFSET(EXHAUST_EXHAUST_FLOW,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F11/F16</f>
+        <f>1+FORECAST(F7,OFFSET(EXHAUST_EXHAUST_FLOW,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F11</f>
         <v/>
       </c>
       <c r="G32" s="11">
-        <f>1+FORECAST(G7,OFFSET(EXHAUST_EXHAUST_FLOW,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G11/G16</f>
+        <f>1+FORECAST(G7,OFFSET(EXHAUST_EXHAUST_FLOW,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G11</f>
         <v/>
       </c>
       <c r="H32" s="11">
-        <f>1+FORECAST(H7,OFFSET(EXHAUST_EXHAUST_FLOW,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H11/H16</f>
+        <f>1+FORECAST(H7,OFFSET(EXHAUST_EXHAUST_FLOW,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H11</f>
         <v/>
       </c>
     </row>
@@ -1656,23 +1656,23 @@
         </is>
       </c>
       <c r="D41" s="10">
-        <f>ISO_EXHAUST_TEMP_C+FORECAST(D7,OFFSET(T_EXHAUST_TEMP,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))+FORECAST(D7,OFFSET(RH_EXHAUST_TEMP,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*(D9/100-0.6)+FORECAST(D7,OFFSET(INLET_EXHAUST_TEMP,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D10/D16+FORECAST(D7,OFFSET(EXHAUST_EXHAUST_TEMP,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D11/D16</f>
+        <f>ISO_EXHAUST_TEMP_C+FORECAST(D7,OFFSET(T_EXHAUST_TEMP,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))+FORECAST(D7,OFFSET(RH_EXHAUST_TEMP,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*(D9/100-0.6)+FORECAST(D7,OFFSET(INLET_EXHAUST_TEMP,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D10+FORECAST(D7,OFFSET(EXHAUST_EXHAUST_TEMP,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(D7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*D11</f>
         <v/>
       </c>
       <c r="E41" s="10">
-        <f>ISO_EXHAUST_TEMP_C+FORECAST(E7,OFFSET(T_EXHAUST_TEMP,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))+FORECAST(E7,OFFSET(RH_EXHAUST_TEMP,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*(E9/100-0.6)+FORECAST(E7,OFFSET(INLET_EXHAUST_TEMP,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E10/E16+FORECAST(E7,OFFSET(EXHAUST_EXHAUST_TEMP,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E11/E16</f>
+        <f>ISO_EXHAUST_TEMP_C+FORECAST(E7,OFFSET(T_EXHAUST_TEMP,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))+FORECAST(E7,OFFSET(RH_EXHAUST_TEMP,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*(E9/100-0.6)+FORECAST(E7,OFFSET(INLET_EXHAUST_TEMP,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E10+FORECAST(E7,OFFSET(EXHAUST_EXHAUST_TEMP,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(E7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*E11</f>
         <v/>
       </c>
       <c r="F41" s="10">
-        <f>ISO_EXHAUST_TEMP_C+FORECAST(F7,OFFSET(T_EXHAUST_TEMP,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))+FORECAST(F7,OFFSET(RH_EXHAUST_TEMP,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*(F9/100-0.6)+FORECAST(F7,OFFSET(INLET_EXHAUST_TEMP,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F10/F16+FORECAST(F7,OFFSET(EXHAUST_EXHAUST_TEMP,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F11/F16</f>
+        <f>ISO_EXHAUST_TEMP_C+FORECAST(F7,OFFSET(T_EXHAUST_TEMP,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))+FORECAST(F7,OFFSET(RH_EXHAUST_TEMP,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*(F9/100-0.6)+FORECAST(F7,OFFSET(INLET_EXHAUST_TEMP,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F10+FORECAST(F7,OFFSET(EXHAUST_EXHAUST_TEMP,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(F7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*F11</f>
         <v/>
       </c>
       <c r="G41" s="10">
-        <f>ISO_EXHAUST_TEMP_C+FORECAST(G7,OFFSET(T_EXHAUST_TEMP,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))+FORECAST(G7,OFFSET(RH_EXHAUST_TEMP,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*(G9/100-0.6)+FORECAST(G7,OFFSET(INLET_EXHAUST_TEMP,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G10/G16+FORECAST(G7,OFFSET(EXHAUST_EXHAUST_TEMP,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G11/G16</f>
+        <f>ISO_EXHAUST_TEMP_C+FORECAST(G7,OFFSET(T_EXHAUST_TEMP,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))+FORECAST(G7,OFFSET(RH_EXHAUST_TEMP,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*(G9/100-0.6)+FORECAST(G7,OFFSET(INLET_EXHAUST_TEMP,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G10+FORECAST(G7,OFFSET(EXHAUST_EXHAUST_TEMP,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(G7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*G11</f>
         <v/>
       </c>
       <c r="H41" s="10">
-        <f>ISO_EXHAUST_TEMP_C+FORECAST(H7,OFFSET(T_EXHAUST_TEMP,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))+FORECAST(H7,OFFSET(RH_EXHAUST_TEMP,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*(H9/100-0.6)+FORECAST(H7,OFFSET(INLET_EXHAUST_TEMP,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H10/H16+FORECAST(H7,OFFSET(EXHAUST_EXHAUST_TEMP,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H11/H16</f>
+        <f>ISO_EXHAUST_TEMP_C+FORECAST(H7,OFFSET(T_EXHAUST_TEMP,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))+FORECAST(H7,OFFSET(RH_EXHAUST_TEMP,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*(H9/100-0.6)+FORECAST(H7,OFFSET(INLET_EXHAUST_TEMP,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H10+FORECAST(H7,OFFSET(EXHAUST_EXHAUST_TEMP,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1),OFFSET(T_GRID,MIN(IFERROR(MATCH(H7,T_GRID,1),1),ROWS(T_GRID)-1)-1,0,2,1))*H11</f>
         <v/>
       </c>
     </row>
@@ -1845,56 +1845,56 @@
         <v>-20</v>
       </c>
       <c r="B2" s="14" t="n">
-        <v>1.335155971261992</v>
+        <v>1.212097329432471</v>
       </c>
       <c r="C2" s="14" t="n">
-        <v>0.9252690468069954</v>
+        <v>0.9417371049535747</v>
       </c>
       <c r="D2" s="14" t="n">
-        <v>1.243493019066825</v>
+        <v>1.185894787887593</v>
       </c>
       <c r="E2" s="14" t="n">
-        <v>-53.81608251948421</v>
+        <v>-63.21575998382207</v>
       </c>
       <c r="F2" s="14" t="n">
-        <v>-0.0005691042480156882</v>
+        <v>0.000189921131383774</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>0.0002837820183797899</v>
+        <v>0.0001747295933695943</v>
       </c>
       <c r="H2" s="14" t="n">
-        <v>-0.0005717874973342139</v>
+        <v>-0.0002593435016833122</v>
       </c>
       <c r="I2" s="14" t="n">
-        <v>-0.09598326718617045</v>
+        <v>0.02701613123046324</v>
       </c>
       <c r="J2" s="14" t="n">
-        <v>-0.001391168431232983</v>
+        <v>-0.00171712055432759</v>
       </c>
       <c r="K2" s="14" t="n">
-        <v>0.0004717592400200144</v>
+        <v>0.0006141319146418641</v>
       </c>
       <c r="L2" s="14" t="n">
-        <v>-0.0009864248851135476</v>
+        <v>-0.001190167748707101</v>
       </c>
       <c r="M2" s="14" t="n">
-        <v>0.1760327871405025</v>
+        <v>0.2188550985440088</v>
       </c>
       <c r="N2" s="14" t="n">
-        <v>-0.0004020530733407966</v>
+        <v>-0.000552006951091936</v>
       </c>
       <c r="O2" s="14" t="n">
-        <v>0.0004681141080733867</v>
+        <v>0.0006428174770368316</v>
       </c>
       <c r="P2" s="14" t="n">
-        <v>5.016650947465988e-07</v>
+        <v>4.120848032738782e-07</v>
       </c>
       <c r="Q2" s="14" t="n">
-        <v>0.1738631345204203</v>
+        <v>0.2275014921691445</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>gas generator speed</t>
+          <t>gas generator corrected speed</t>
         </is>
       </c>
     </row>
@@ -1903,56 +1903,56 @@
         <v>-15</v>
       </c>
       <c r="B3" s="14" t="n">
-        <v>1.300702480144624</v>
+        <v>1.225901920331932</v>
       </c>
       <c r="C3" s="14" t="n">
-        <v>0.9327281922253925</v>
+        <v>0.9441548304886096</v>
       </c>
       <c r="D3" s="14" t="n">
-        <v>1.212675462033141</v>
+        <v>1.174650113677684</v>
       </c>
       <c r="E3" s="14" t="n">
-        <v>-43.8191477404165</v>
+        <v>-47.27497772473828</v>
       </c>
       <c r="F3" s="14" t="n">
-        <v>-0.0008642398712572423</v>
+        <v>0.000285510363491498</v>
       </c>
       <c r="G3" s="14" t="n">
-        <v>0.0004380236182299227</v>
+        <v>0.0002750738751507021</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>-0.0008721757412085889</v>
+        <v>-0.0003947609406326594</v>
       </c>
       <c r="I3" s="14" t="n">
-        <v>-0.1437783627650333</v>
+        <v>0.04547832921029264</v>
       </c>
       <c r="J3" s="14" t="n">
-        <v>-0.001395417524612137</v>
+        <v>-0.001711363208186354</v>
       </c>
       <c r="K3" s="14" t="n">
-        <v>0.0004789034783387551</v>
+        <v>0.0006086279479197169</v>
       </c>
       <c r="L3" s="14" t="n">
-        <v>-0.0009864257935182173</v>
+        <v>-0.00118967557532117</v>
       </c>
       <c r="M3" s="14" t="n">
-        <v>0.1792363238668145</v>
+        <v>0.220728331203361</v>
       </c>
       <c r="N3" s="14" t="n">
-        <v>-0.0004062632949146366</v>
+        <v>-0.0005475490756730735</v>
       </c>
       <c r="O3" s="14" t="n">
-        <v>0.0004752381050274626</v>
+        <v>0.0006383073674975702</v>
       </c>
       <c r="P3" s="14" t="n">
-        <v>5.007219043808557e-07</v>
+        <v>4.425793644452656e-07</v>
       </c>
       <c r="Q3" s="14" t="n">
-        <v>0.1770374477214455</v>
+        <v>0.2299165794476767</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>gas generator speed</t>
+          <t>gas generator corrected speed</t>
         </is>
       </c>
     </row>
@@ -1961,56 +1961,56 @@
         <v>-10</v>
       </c>
       <c r="B4" s="14" t="n">
-        <v>1.267725650843293</v>
+        <v>1.239341900922081</v>
       </c>
       <c r="C4" s="14" t="n">
-        <v>0.9402859962454216</v>
+        <v>0.9468000769665297</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>1.18306691941724</v>
+        <v>1.163690568505592</v>
       </c>
       <c r="E4" s="14" t="n">
-        <v>-33.78740557458298</v>
+        <v>-31.27904191244716</v>
       </c>
       <c r="F4" s="14" t="n">
-        <v>-0.001289619285298176</v>
+        <v>0.0004218237198164983</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>0.0006640617034990256</v>
+        <v>0.0004245405739387977</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>-0.001306906288256758</v>
+        <v>-0.0005902515835989226</v>
       </c>
       <c r="I4" s="14" t="n">
-        <v>-0.2115679017728098</v>
+        <v>0.07450642227619635</v>
       </c>
       <c r="J4" s="14" t="n">
-        <v>-0.001399596689727202</v>
+        <v>-0.001705734114056737</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>0.0004860397754772805</v>
+        <v>0.0006033418579780629</v>
       </c>
       <c r="L4" s="14" t="n">
-        <v>-0.0009864304797140735</v>
+        <v>-0.001189094216437867</v>
       </c>
       <c r="M4" s="14" t="n">
-        <v>0.1824735347481919</v>
+        <v>0.2225284862147305</v>
       </c>
       <c r="N4" s="14" t="n">
-        <v>-0.0004104034122578723</v>
+        <v>-0.0005433159128026737</v>
       </c>
       <c r="O4" s="14" t="n">
-        <v>0.0004823546372614582</v>
+        <v>0.0006340276435050607</v>
       </c>
       <c r="P4" s="14" t="n">
-        <v>4.959709033271408e-07</v>
+        <v>4.736801334597733e-07</v>
       </c>
       <c r="Q4" s="14" t="n">
-        <v>0.1802454174107425</v>
+        <v>0.2322717333556602</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>gas generator speed</t>
+          <t>gas generator corrected speed</t>
         </is>
       </c>
     </row>
@@ -2019,52 +2019,52 @@
         <v>-5</v>
       </c>
       <c r="B5" s="14" t="n">
-        <v>1.231487873085713</v>
+        <v>1.212976328187749</v>
       </c>
       <c r="C5" s="14" t="n">
-        <v>0.9484730843523687</v>
+        <v>0.952231679901489</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>1.152747052385822</v>
+        <v>1.1408021984244</v>
       </c>
       <c r="E5" s="14" t="n">
-        <v>-24.34127314993236</v>
+        <v>-23.49690751594346</v>
       </c>
       <c r="F5" s="14" t="n">
-        <v>0.002472679504958275</v>
+        <v>0.002072431032358455</v>
       </c>
       <c r="G5" s="14" t="n">
-        <v>0.0003552555359570275</v>
+        <v>0.0004740513555447998</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>-8.578180258360867e-05</v>
+        <v>-0.0003560159825396862</v>
       </c>
       <c r="I5" s="14" t="n">
-        <v>0.4107696508241361</v>
+        <v>0.4420059622935923</v>
       </c>
       <c r="J5" s="14" t="n">
-        <v>-0.001536920355994321</v>
+        <v>-0.001790188511238522</v>
       </c>
       <c r="K5" s="14" t="n">
-        <v>0.0005143791244374392</v>
+        <v>0.0006108051059315936</v>
       </c>
       <c r="L5" s="14" t="n">
-        <v>-0.001042372566001456</v>
+        <v>-0.001205105308054186</v>
       </c>
       <c r="M5" s="14" t="n">
-        <v>0.1640164609251087</v>
+        <v>0.1939469799534549</v>
       </c>
       <c r="N5" s="14" t="n">
-        <v>-0.000548352542542882</v>
+        <v>-0.0006530674167267319</v>
       </c>
       <c r="O5" s="14" t="n">
-        <v>0.0005114542358961091</v>
+        <v>0.0006357253664098983</v>
       </c>
       <c r="P5" s="14" t="n">
-        <v>-5.592641013635446e-05</v>
+        <v>-4.335591699703342e-05</v>
       </c>
       <c r="Q5" s="14" t="n">
-        <v>0.1619026721825321</v>
+        <v>0.199996420294583</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -2077,52 +2077,52 @@
         <v>0</v>
       </c>
       <c r="B6" s="14" t="n">
-        <v>1.169546078761788</v>
+        <v>1.162140002990242</v>
       </c>
       <c r="C6" s="14" t="n">
-        <v>0.9602076457474391</v>
+        <v>0.9615018212083526</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>1.112667746769416</v>
+        <v>1.107734420866573</v>
       </c>
       <c r="E6" s="14" t="n">
-        <v>-18.51210073989398</v>
+        <v>-18.37513855312204</v>
       </c>
       <c r="F6" s="14" t="n">
-        <v>0.003659115032547931</v>
+        <v>0.003402588857325272</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>0.0004651654411378912</v>
+        <v>0.0005347569952256938</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>-9.853524782378449e-05</v>
+        <v>-0.000267677719805966</v>
       </c>
       <c r="I6" s="14" t="n">
-        <v>0.5762483960992313</v>
+        <v>0.5897056182105114</v>
       </c>
       <c r="J6" s="14" t="n">
-        <v>-0.001560517326160122</v>
+        <v>-0.001759932918196642</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>0.0005336433548895494</v>
+        <v>0.0006109425794765666</v>
       </c>
       <c r="L6" s="14" t="n">
-        <v>-0.001048214918213178</v>
+        <v>-0.001175045167477332</v>
       </c>
       <c r="M6" s="14" t="n">
-        <v>0.1675187036901548</v>
+        <v>0.1914494103415677</v>
       </c>
       <c r="N6" s="14" t="n">
-        <v>-0.0005719348073886724</v>
+        <v>-0.0006599398860234544</v>
       </c>
       <c r="O6" s="14" t="n">
-        <v>0.0005308095779901511</v>
+        <v>0.0006278116158717796</v>
       </c>
       <c r="P6" s="14" t="n">
-        <v>-6.18284983354676e-05</v>
+        <v>-5.844204017256218e-05</v>
       </c>
       <c r="Q6" s="14" t="n">
-        <v>0.1653819075860656</v>
+        <v>0.1949604818463831</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -2135,52 +2135,52 @@
         <v>5</v>
       </c>
       <c r="B7" s="14" t="n">
-        <v>1.110357364482509</v>
+        <v>1.106701509976154</v>
       </c>
       <c r="C7" s="14" t="n">
-        <v>0.9726638785112107</v>
+        <v>0.9732602705808414</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>1.073891842107071</v>
+        <v>1.071377341166532</v>
       </c>
       <c r="E7" s="14" t="n">
-        <v>-12.52311175820978</v>
+        <v>-12.50488672747463</v>
       </c>
       <c r="F7" s="14" t="n">
-        <v>0.00533658613894034</v>
+        <v>0.005190435713255473</v>
       </c>
       <c r="G7" s="14" t="n">
-        <v>0.000588922758077259</v>
+        <v>0.0006159265061110487</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>-0.000102852783277088</v>
+        <v>-0.0001958865999598064</v>
       </c>
       <c r="I7" s="14" t="n">
-        <v>0.7946743053282717</v>
+        <v>0.7928894242227595</v>
       </c>
       <c r="J7" s="14" t="n">
-        <v>-0.001585803624516228</v>
+        <v>-0.001712123534572268</v>
       </c>
       <c r="K7" s="14" t="n">
-        <v>0.0005541172034427913</v>
+        <v>0.000606036276299535</v>
       </c>
       <c r="L7" s="14" t="n">
-        <v>-0.001054684742133139</v>
+        <v>-0.001132216214020744</v>
       </c>
       <c r="M7" s="14" t="n">
-        <v>0.1711896403406513</v>
+        <v>0.1870274764413125</v>
       </c>
       <c r="N7" s="14" t="n">
-        <v>-0.0005972110287659955</v>
+        <v>-0.0006563391794443643</v>
       </c>
       <c r="O7" s="14" t="n">
-        <v>0.0005513986835631769</v>
+        <v>0.0006155948041738113</v>
       </c>
       <c r="P7" s="14" t="n">
-        <v>-6.836663170796402e-05</v>
+        <v>-6.706228063020687e-05</v>
       </c>
       <c r="Q7" s="14" t="n">
-        <v>0.1690310546700903</v>
+        <v>0.1883131605385734</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
@@ -2193,52 +2193,52 @@
         <v>10</v>
       </c>
       <c r="B8" s="14" t="n">
-        <v>1.053856805541576</v>
+        <v>1.051555194239657</v>
       </c>
       <c r="C8" s="14" t="n">
-        <v>0.9859057393337989</v>
+        <v>0.9864146291027306</v>
       </c>
       <c r="D8" s="14" t="n">
-        <v>1.036355093337257</v>
+        <v>1.034773760588782</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>-6.35810027507398</v>
+        <v>-6.27625124283918</v>
       </c>
       <c r="F8" s="14" t="n">
-        <v>0.007676611975332574</v>
+        <v>0.007480521204586399</v>
       </c>
       <c r="G8" s="14" t="n">
-        <v>0.0007170252454227454</v>
+        <v>0.0007532644651522868</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>-9.028594759498202e-05</v>
+        <v>-0.0002148506930969151</v>
       </c>
       <c r="I8" s="14" t="n">
-        <v>1.078038343272965</v>
+        <v>1.077803391001263</v>
       </c>
       <c r="J8" s="14" t="n">
-        <v>-0.001612921476433409</v>
+        <v>-0.001655010062419213</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>0.0005758923160186992</v>
+        <v>0.0005977520548465585</v>
       </c>
       <c r="L8" s="14" t="n">
-        <v>-0.001061846745050555</v>
+        <v>-0.001083283509312694</v>
       </c>
       <c r="M8" s="14" t="n">
-        <v>0.1750376975629365</v>
+        <v>0.1814874344207624</v>
       </c>
       <c r="N8" s="14" t="n">
-        <v>-0.0006243247499745535</v>
+        <v>-0.0006444838304763348</v>
       </c>
       <c r="O8" s="14" t="n">
-        <v>0.0005733175625904575</v>
+        <v>0.0006006154070857284</v>
       </c>
       <c r="P8" s="14" t="n">
-        <v>-7.560687498355098e-05</v>
+        <v>-6.995605619833103e-05</v>
       </c>
       <c r="Q8" s="14" t="n">
-        <v>0.1728589515844942</v>
+        <v>0.1808133061540366</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
@@ -2251,52 +2251,52 @@
         <v>15</v>
       </c>
       <c r="B9" s="14" t="n">
-        <v>1.000000000000009</v>
+        <v>1.000000000000001</v>
       </c>
       <c r="C9" s="14" t="n">
-        <v>0.9999999999999961</v>
+        <v>0.9999999999999994</v>
       </c>
       <c r="D9" s="14" t="n">
-        <v>1.000000000000008</v>
+        <v>1</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>-1.70530256582424e-12</v>
+        <v>1.13686837721616e-13</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>0.01089919505258998</v>
+        <v>0.01030306336408385</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>0.0008318665163371212</v>
+        <v>0.001003884569025062</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>-4.837621730615597e-05</v>
+        <v>-0.0004296140430416784</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>1.439538676354346</v>
+        <v>1.480001291751213</v>
       </c>
       <c r="J9" s="14" t="n">
-        <v>-0.00164201201836476</v>
+        <v>-0.001594740276336782</v>
       </c>
       <c r="K9" s="14" t="n">
-        <v>0.0005990565412248054</v>
+        <v>0.0005874078026104914</v>
       </c>
       <c r="L9" s="14" t="n">
-        <v>-0.00106976798725026</v>
+        <v>-0.001033138216543966</v>
       </c>
       <c r="M9" s="14" t="n">
-        <v>0.1790685158543852</v>
+        <v>0.1754505536973397</v>
       </c>
       <c r="N9" s="14" t="n">
-        <v>-0.0006534187141628573</v>
+        <v>-0.0006265276821636827</v>
       </c>
       <c r="O9" s="14" t="n">
-        <v>0.0005966591059260783</v>
+        <v>0.0005840468008178247</v>
       </c>
       <c r="P9" s="14" t="n">
-        <v>-8.361782150340886e-05</v>
+        <v>-6.815953937851064e-05</v>
       </c>
       <c r="Q9" s="14" t="n">
-        <v>0.1768717372715537</v>
+        <v>0.1730244662981568</v>
       </c>
       <c r="R9" t="inlineStr">
         <is>
@@ -2309,52 +2309,52 @@
         <v>20</v>
       </c>
       <c r="B10" s="14" t="n">
-        <v>0.9487636650345469</v>
+        <v>0.9536854314126401</v>
       </c>
       <c r="C10" s="14" t="n">
-        <v>1.015014523522647</v>
+        <v>1.013322431137116</v>
       </c>
       <c r="D10" s="14" t="n">
-        <v>0.9647761829826441</v>
+        <v>0.968101142639526</v>
       </c>
       <c r="E10" s="14" t="n">
-        <v>6.568747551123352</v>
+        <v>6.130409711943457</v>
       </c>
       <c r="F10" s="14" t="n">
-        <v>0.01528265622284213</v>
+        <v>0.01388544312751843</v>
       </c>
       <c r="G10" s="14" t="n">
-        <v>0.0009045139968295041</v>
+        <v>0.001370941864508188</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>4.032385461953866e-05</v>
+        <v>-0.0008424785922547998</v>
       </c>
       <c r="I10" s="14" t="n">
-        <v>1.893332371230485</v>
+        <v>2.022135293288064</v>
       </c>
       <c r="J10" s="14" t="n">
-        <v>-0.00167320805287697</v>
+        <v>-0.001538191763247129</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>0.000623687712147249</v>
+        <v>0.0005770825850313272</v>
       </c>
       <c r="L10" s="14" t="n">
-        <v>-0.001078515665245603</v>
+        <v>-0.0009866893037224136</v>
       </c>
       <c r="M10" s="14" t="n">
-        <v>0.183283274397354</v>
+        <v>0.1696612269751313</v>
       </c>
       <c r="N10" s="14" t="n">
-        <v>-0.0006846276725370302</v>
+        <v>-0.0006076505898147885</v>
       </c>
       <c r="O10" s="14" t="n">
-        <v>0.0006215068815850704</v>
+        <v>0.0005679173185544292</v>
       </c>
       <c r="P10" s="14" t="n">
-        <v>-9.246837333432409e-05</v>
+        <v>-6.49729975907108e-05</v>
       </c>
       <c r="Q10" s="14" t="n">
-        <v>0.1810711796244141</v>
+        <v>0.1656553575667795</v>
       </c>
       <c r="R10" t="inlineStr">
         <is>
@@ -2367,52 +2367,52 @@
         <v>25</v>
       </c>
       <c r="B11" s="14" t="n">
-        <v>0.9001460169167425</v>
+        <v>0.9116788741121965</v>
       </c>
       <c r="C11" s="14" t="n">
-        <v>1.031015762314368</v>
+        <v>1.026566023638844</v>
       </c>
       <c r="D11" s="14" t="n">
-        <v>0.9306407203388833</v>
+        <v>0.9384457809779646</v>
       </c>
       <c r="E11" s="14" t="n">
-        <v>13.36566989507196</v>
+        <v>12.19677988366993</v>
       </c>
       <c r="F11" s="14" t="n">
-        <v>0.02117408643700421</v>
+        <v>0.01879301683888076</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>0.0008909683524926578</v>
+        <v>0.001739974313207101</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>0.0001991098900121296</v>
+        <v>-0.001276117194062953</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>2.454263683956128</v>
+        <v>2.697482549130731</v>
       </c>
       <c r="J11" s="14" t="n">
-        <v>-0.001706624683850858</v>
+        <v>-0.00148951348533378</v>
       </c>
       <c r="K11" s="14" t="n">
-        <v>0.0006498451929417436</v>
+        <v>0.0005685871447145904</v>
       </c>
       <c r="L11" s="14" t="n">
-        <v>-0.001088154305489066</v>
+        <v>-0.0009463818876066805</v>
       </c>
       <c r="M11" s="14" t="n">
-        <v>0.1876764437042084</v>
+        <v>0.1646006928839256</v>
       </c>
       <c r="N11" s="14" t="n">
-        <v>-0.00071806913420036</v>
+        <v>-0.000593122661945544</v>
       </c>
       <c r="O11" s="14" t="n">
-        <v>0.0006479266607006167</v>
+        <v>0.000553972707102508</v>
       </c>
       <c r="P11" s="14" t="n">
-        <v>-0.0001022249505817847</v>
+        <v>-6.407678336951525e-05</v>
       </c>
       <c r="Q11" s="14" t="n">
-        <v>0.1854524249338965</v>
+        <v>0.1591526918186764</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2425,52 +2425,52 @@
         <v>30</v>
       </c>
       <c r="B12" s="14" t="n">
-        <v>0.8541666375678799</v>
+        <v>0.8726491555115999</v>
       </c>
       <c r="C12" s="14" t="n">
-        <v>1.04806545967766</v>
+        <v>1.040197703719112</v>
       </c>
       <c r="D12" s="14" t="n">
-        <v>0.8975582191731517</v>
+        <v>0.9101169472256658</v>
       </c>
       <c r="E12" s="14" t="n">
-        <v>20.40759978061635</v>
+        <v>18.35474676112051</v>
       </c>
       <c r="F12" s="14" t="n">
-        <v>0.0290000095035467</v>
+        <v>0.02552565786988288</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>0.0007280813026981693</v>
+        <v>0.002024128583872154</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>0.0004577359329655641</v>
+        <v>-0.001641574095792873</v>
       </c>
       <c r="I12" s="14" t="n">
-        <v>3.137666438291944</v>
+        <v>3.514875222551079</v>
       </c>
       <c r="J12" s="14" t="n">
-        <v>-0.001742349994130616</v>
+        <v>-0.001446353273168094</v>
       </c>
       <c r="K12" s="14" t="n">
-        <v>0.000677559726232364</v>
+        <v>0.0005614014526621935</v>
       </c>
       <c r="L12" s="14" t="n">
-        <v>-0.001098743667782387</v>
+        <v>-0.0009103553795922825</v>
       </c>
       <c r="M12" s="14" t="n">
-        <v>0.1922330069097143</v>
+        <v>0.1600253468530582</v>
       </c>
       <c r="N12" s="14" t="n">
-        <v>-0.000753834409218688</v>
+        <v>-0.0005822964053629346</v>
       </c>
       <c r="O12" s="14" t="n">
-        <v>0.0006759562734873315</v>
+        <v>0.0005417326797683475</v>
       </c>
       <c r="P12" s="14" t="n">
-        <v>-0.0001129495385753304</v>
+        <v>-6.527990722394466e-05</v>
       </c>
       <c r="Q12" s="14" t="n">
-        <v>0.1900012173821369</v>
+        <v>0.1532829770020817</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2483,52 +2483,52 @@
         <v>35</v>
       </c>
       <c r="B13" s="14" t="n">
-        <v>0.8108651361636405</v>
+        <v>0.8355959937664581</v>
       </c>
       <c r="C13" s="14" t="n">
-        <v>1.066216874634438</v>
+        <v>1.054692102762172</v>
       </c>
       <c r="D13" s="14" t="n">
-        <v>0.8655001119592822</v>
+        <v>0.8823899642537609</v>
       </c>
       <c r="E13" s="14" t="n">
-        <v>27.70995677867393</v>
+        <v>24.75002715587414</v>
       </c>
       <c r="F13" s="14" t="n">
-        <v>0.03927746823983532</v>
+        <v>0.03482833889981082</v>
       </c>
       <c r="G13" s="14" t="n">
-        <v>0.0003291558679296361</v>
+        <v>0.002042454854440197</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>0.0008530757876170331</v>
+        <v>-0.001742816518244103</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>3.959351202440757</v>
+        <v>4.464380322816055</v>
       </c>
       <c r="J13" s="14" t="n">
-        <v>-0.001780444647149142</v>
+        <v>-0.001407315301703855</v>
       </c>
       <c r="K13" s="14" t="n">
-        <v>0.0007068250761252525</v>
+        <v>0.0005552693240110834</v>
       </c>
       <c r="L13" s="14" t="n">
-        <v>-0.001110342338413822</v>
+        <v>-0.0008774576824767668</v>
       </c>
       <c r="M13" s="14" t="n">
-        <v>0.1969257561408881</v>
+        <v>0.1557869173917084</v>
       </c>
       <c r="N13" s="14" t="n">
-        <v>-0.0007919895526558251</v>
+        <v>-0.0005750841109755374</v>
       </c>
       <c r="O13" s="14" t="n">
-        <v>0.0007055976441259513</v>
+        <v>0.0005309891070879068</v>
       </c>
       <c r="P13" s="14" t="n">
-        <v>-0.0001247039929677314</v>
+        <v>-6.86978375142964e-05</v>
       </c>
       <c r="Q13" s="14" t="n">
-        <v>0.1946912499199243</v>
+        <v>0.1479101247068638</v>
       </c>
       <c r="R13" t="inlineStr">
         <is>
@@ -2541,52 +2541,52 @@
         <v>40</v>
       </c>
       <c r="B14" s="14" t="n">
-        <v>0.7702968186178835</v>
+        <v>0.7996664020916082</v>
       </c>
       <c r="C14" s="14" t="n">
-        <v>1.085511838828136</v>
+        <v>1.070597054013051</v>
       </c>
       <c r="D14" s="14" t="n">
-        <v>0.8344419078266418</v>
+        <v>0.8546189152860467</v>
       </c>
       <c r="E14" s="14" t="n">
-        <v>35.2862531891509</v>
+        <v>31.53579488874504</v>
       </c>
       <c r="F14" s="14" t="n">
-        <v>0.05262977678119753</v>
+        <v>0.04785844709982542</v>
       </c>
       <c r="G14" s="14" t="n">
-        <v>-0.0004223179328935722</v>
+        <v>0.001432690660903316</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>0.001432552188491042</v>
+        <v>-0.001180044174686553</v>
       </c>
       <c r="I14" s="14" t="n">
-        <v>4.935624746388612</v>
+        <v>5.496453570335879</v>
       </c>
       <c r="J14" s="14" t="n">
-        <v>-0.001820982010165379</v>
+        <v>-0.001371840218466992</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>0.0007376052844477066</v>
+        <v>0.0005502224361003696</v>
       </c>
       <c r="L14" s="14" t="n">
-        <v>-0.001123034553118407</v>
+        <v>-0.0008471030388114345</v>
       </c>
       <c r="M14" s="14" t="n">
-        <v>0.2017153970590698</v>
+        <v>0.1518229267625884</v>
       </c>
       <c r="N14" s="14" t="n">
-        <v>-0.0008326206463469334</v>
+        <v>-0.0005720238260684809</v>
       </c>
       <c r="O14" s="14" t="n">
-        <v>0.0007368263643812403</v>
+        <v>0.0005218215150912366</v>
       </c>
       <c r="P14" s="14" t="n">
-        <v>-0.000137579883874401</v>
+        <v>-7.480559273275937e-05</v>
       </c>
       <c r="Q14" s="14" t="n">
-        <v>0.1994846455654124</v>
+        <v>0.1429834004160421</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
@@ -2599,52 +2599,52 @@
         <v>45</v>
       </c>
       <c r="B15" s="14" t="n">
-        <v>0.7325202398482688</v>
+        <v>0.7642836934559698</v>
       </c>
       <c r="C15" s="14" t="n">
-        <v>1.105982984005574</v>
+        <v>1.088463559156613</v>
       </c>
       <c r="D15" s="14" t="n">
-        <v>0.804354884676587</v>
+        <v>0.8263273704487484</v>
       </c>
       <c r="E15" s="14" t="n">
-        <v>43.14868727324574</v>
+        <v>38.85197316078029</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>0.06983217431650399</v>
+        <v>0.0651647828172571</v>
       </c>
       <c r="G15" s="14" t="n">
-        <v>-0.001691520283254659</v>
+        <v>4.782515702069531e-05</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>0.002275478920821667</v>
+        <v>2.475489422431432e-06</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>6.081246925355686</v>
+        <v>6.635336379773852</v>
       </c>
       <c r="J15" s="14" t="n">
-        <v>-0.001864243236677761</v>
+        <v>-0.001336511079546952</v>
       </c>
       <c r="K15" s="14" t="n">
-        <v>0.0007699095803217675</v>
+        <v>0.000545047881461863</v>
       </c>
       <c r="L15" s="14" t="n">
-        <v>-0.001137044182588025</v>
+        <v>-0.0008170216504841659</v>
       </c>
       <c r="M15" s="14" t="n">
-        <v>0.2065645755627088</v>
+        <v>0.1477478830025461</v>
       </c>
       <c r="N15" s="14" t="n">
-        <v>-0.0008760499239232303</v>
+        <v>-0.0005703745227394547</v>
       </c>
       <c r="O15" s="14" t="n">
-        <v>0.0007696775955187201</v>
+        <v>0.0005130381641906144</v>
       </c>
       <c r="P15" s="14" t="n">
-        <v>-0.0001518252394354583</v>
+        <v>-8.197086231601679e-05</v>
       </c>
       <c r="Q15" s="14" t="n">
-        <v>0.2043479520885648</v>
+        <v>0.1381262823509678</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
@@ -2657,52 +2657,52 @@
         <v>50</v>
       </c>
       <c r="B16" s="14" t="n">
-        <v>0.6975602935444133</v>
+        <v>0.7300827843602042</v>
       </c>
       <c r="C16" s="14" t="n">
-        <v>1.12767576035671</v>
+        <v>1.108242071619398</v>
       </c>
       <c r="D16" s="14" t="n">
-        <v>0.7751812254382082</v>
+        <v>0.7978320043038403</v>
       </c>
       <c r="E16" s="14" t="n">
-        <v>51.31272491018137</v>
+        <v>46.67931371908094</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>0.09202857508044705</v>
+        <v>0.08663815420074719</v>
       </c>
       <c r="G16" s="14" t="n">
-        <v>-0.00378891701694551</v>
+        <v>-0.001977490806408816</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>0.003617504670806056</v>
+        <v>0.001310462514362485</v>
       </c>
       <c r="I16" s="14" t="n">
-        <v>7.390376305376435</v>
+        <v>7.990709746997974</v>
       </c>
       <c r="J16" s="14" t="n">
-        <v>-0.001911513693648213</v>
+        <v>-0.001297244670275575</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>0.0008041423343746412</v>
+        <v>0.0005378405163906668</v>
       </c>
       <c r="L16" s="14" t="n">
-        <v>-0.001153188297366022</v>
+        <v>-0.0007849228166387277</v>
       </c>
       <c r="M16" s="14" t="n">
-        <v>0.2115132010286402</v>
+        <v>0.1430976903829446</v>
       </c>
       <c r="N16" s="14" t="n">
-        <v>-0.0009237249690303393</v>
+        <v>-0.0005657438355343138</v>
       </c>
       <c r="O16" s="14" t="n">
-        <v>0.0008046472238219783</v>
+        <v>0.0005028639289050785</v>
       </c>
       <c r="P16" s="14" t="n">
-        <v>-0.0001683550818976937</v>
+        <v>-8.743496721456604e-05</v>
       </c>
       <c r="Q16" s="14" t="n">
-        <v>0.2093374692861016</v>
+        <v>0.1329079477731011</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
@@ -2741,16 +2741,16 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>12.9</v>
+        <v>12.88868202588779</v>
       </c>
       <c r="B21" t="n">
-        <v>10294.00000000002</v>
+        <v>10297.96992889297</v>
       </c>
       <c r="C21" t="n">
-        <v>40.00000000000001</v>
+        <v>39.97369050857318</v>
       </c>
       <c r="D21" t="n">
-        <v>550.1991534718409</v>
+        <v>550.4464565636417</v>
       </c>
     </row>
   </sheetData>
@@ -2828,7 +2828,7 @@
         </is>
       </c>
       <c r="D5" s="17" t="n">
-        <v>12.9</v>
+        <v>12.88868202588782</v>
       </c>
       <c r="E5" s="17">
         <f>'Site tool'!D36</f>
@@ -2851,7 +2851,7 @@
         </is>
       </c>
       <c r="D6" s="19" t="n">
-        <v>10294.00000000002</v>
+        <v>10297.96992889294</v>
       </c>
       <c r="E6" s="19">
         <f>'Site tool'!D37</f>
@@ -2874,7 +2874,7 @@
         </is>
       </c>
       <c r="D7" s="17" t="n">
-        <v>40.00000000000001</v>
+        <v>39.97369050857321</v>
       </c>
       <c r="E7" s="17">
         <f>'Site tool'!D40</f>
@@ -2897,7 +2897,7 @@
         </is>
       </c>
       <c r="D8" s="20" t="n">
-        <v>550.1991534718409</v>
+        <v>550.4464565636417</v>
       </c>
       <c r="E8" s="20">
         <f>'Site tool'!D41</f>
@@ -2920,7 +2920,7 @@
         </is>
       </c>
       <c r="D9" s="17" t="n">
-        <v>13.26472571011501</v>
+        <v>13.21653842270864</v>
       </c>
       <c r="E9" s="17">
         <f>'Site tool'!E36</f>
@@ -2943,7 +2943,7 @@
         </is>
       </c>
       <c r="D10" s="19" t="n">
-        <v>10285.55048024335</v>
+        <v>10299.91541005129</v>
       </c>
       <c r="E10" s="19">
         <f>'Site tool'!E37</f>
@@ -2966,7 +2966,7 @@
         </is>
       </c>
       <c r="D11" s="17" t="n">
-        <v>40.90699658376359</v>
+        <v>40.81402733007079</v>
       </c>
       <c r="E11" s="17">
         <f>'Site tool'!E40</f>
@@ -2989,7 +2989,7 @@
         </is>
       </c>
       <c r="D12" s="20" t="n">
-        <v>548.0783084270118</v>
+        <v>548.5505142378677</v>
       </c>
       <c r="E12" s="20">
         <f>'Site tool'!E41</f>
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D13" s="17" t="n">
-        <v>8.488995754045042</v>
+        <v>9.00470389973502</v>
       </c>
       <c r="E13" s="17">
         <f>'Site tool'!F36</f>
@@ -3035,7 +3035,7 @@
         </is>
       </c>
       <c r="D14" s="19" t="n">
-        <v>11725.86278882141</v>
+        <v>11416.3237665638</v>
       </c>
       <c r="E14" s="19">
         <f>'Site tool'!F37</f>
@@ -3058,7 +3058,7 @@
         </is>
       </c>
       <c r="D15" s="17" t="n">
-        <v>30.52141677770948</v>
+        <v>31.54778491741571</v>
       </c>
       <c r="E15" s="17">
         <f>'Site tool'!F40</f>
@@ -3081,7 +3081,7 @@
         </is>
       </c>
       <c r="D16" s="20" t="n">
-        <v>598.6244047245948</v>
+        <v>591.6506592619655</v>
       </c>
       <c r="E16" s="20">
         <f>'Site tool'!F41</f>
@@ -3104,7 +3104,7 @@
         </is>
       </c>
       <c r="D17" s="17" t="n">
-        <v>10.54869247461472</v>
+        <v>10.86710387157749</v>
       </c>
       <c r="E17" s="17">
         <f>'Site tool'!G36</f>
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="D18" s="19" t="n">
-        <v>11074.21746685397</v>
+        <v>10939.78049297851</v>
       </c>
       <c r="E18" s="19">
         <f>'Site tool'!G37</f>
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="D19" s="17" t="n">
-        <v>34.95200799323936</v>
+        <v>35.5721193768031</v>
       </c>
       <c r="E19" s="17">
         <f>'Site tool'!G40</f>
@@ -3173,7 +3173,7 @@
         </is>
       </c>
       <c r="D20" s="20" t="n">
-        <v>579.7550550817107</v>
+        <v>576.5609591323389</v>
       </c>
       <c r="E20" s="20">
         <f>'Site tool'!G41</f>
@@ -3196,7 +3196,7 @@
         </is>
       </c>
       <c r="D21" s="17" t="n">
-        <v>13.094553465991</v>
+        <v>12.77989960557742</v>
       </c>
       <c r="E21" s="17">
         <f>'Site tool'!H36</f>
@@ -3219,7 +3219,7 @@
         </is>
       </c>
       <c r="D22" s="19" t="n">
-        <v>9908.158339167248</v>
+        <v>9989.268169034191</v>
       </c>
       <c r="E22" s="19">
         <f>'Site tool'!H37</f>
@@ -3242,7 +3242,7 @@
         </is>
       </c>
       <c r="D23" s="17" t="n">
-        <v>39.11173024484501</v>
+        <v>38.44515474907153</v>
       </c>
       <c r="E23" s="17">
         <f>'Site tool'!H40</f>
@@ -3265,7 +3265,7 @@
         </is>
       </c>
       <c r="D24" s="20" t="n">
-        <v>521.3994261684024</v>
+        <v>524.4320313567752</v>
       </c>
       <c r="E24" s="20">
         <f>'Site tool'!H41</f>
@@ -3348,7 +3348,7 @@
     <row r="9">
       <c r="A9" s="23" t="inlineStr">
         <is>
-          <t>Losses are divided by delta because their effect depends on the loss as a fraction of ambient pressure.</t>
+          <t>Losses are entered at rated flow. The model scales them with dynamic head, which falls with ambient pressure at altitude, so they need no altitude correction.</t>
         </is>
       </c>
     </row>

</xml_diff>